<commit_message>
Chapter 5 project finished
</commit_message>
<xml_diff>
--- a/3_Excel/Chapter_1_Excel_Fundamentals/c1_task_1.xlsx
+++ b/3_Excel/Chapter_1_Excel_Fundamentals/c1_task_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROITBRIDGE_Learning\3_Excel\Chapter_1_Excel_Fundamentals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F48BEA-462D-4CDC-874A-228731858E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E6B8F3-42DB-4E94-A848-E6F3AB7EA6EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">Destination </t>
   </si>
@@ -97,6 +97,15 @@
   </si>
   <si>
     <t>Tax Amount</t>
+  </si>
+  <si>
+    <t>👆 Absolute Reference</t>
+  </si>
+  <si>
+    <t>👆 Mixed Reference</t>
+  </si>
+  <si>
+    <t>👆 Relative Reference</t>
   </si>
 </sst>
 </file>
@@ -105,10 +114,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="174" formatCode="[$-14009]dd\ mmmm\ yyyy;@"/>
-    <numFmt numFmtId="178" formatCode="_ [$₹-449]\ * #,##0.00_ ;_ [$₹-449]\ * \-#,##0.00_ ;_ [$₹-449]\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="[$₹-449]\ #,##0.00"/>
-    <numFmt numFmtId="181" formatCode="[$₹-449]\ #,##0.00;[$₹-449]\ \-#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$-14009]dd\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="_ [$₹-449]\ * #,##0.00_ ;_ [$₹-449]\ * \-#,##0.00_ ;_ [$₹-449]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="[$₹-449]\ #,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$₹-449]\ #,##0.00;[$₹-449]\ \-#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -141,12 +150,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -163,20 +178,21 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="174" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -677,6 +693,17 @@
         <v>21500</v>
       </c>
     </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>17</v>

</xml_diff>